<commit_message>
Improvements after detection of flow deployment error
</commit_message>
<xml_diff>
--- a/docs/Import/FeedbackDeployment_20-09-2026.xlsx
+++ b/docs/Import/FeedbackDeployment_20-09-2026.xlsx
@@ -12453,4 +12453,217 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae75f7d6110eb3c01e30b5864ecce8d9">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" xmlns:ns3="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f758225586994ab2ed7147b7dc97d7e" ns2:_="" ns3:_="">
+    <xsd:import namespace="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
+    <xsd:import namespace="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f28f5036-0c97-4fb2-9995-e6511ad4535b" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="3edfda32-ed56-4dd9-bd64-14fdcb8b12da" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{309b44fd-1af0-4c99-971b-3abc3e199a55}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="d3a2e4d4-5189-48ac-a210-e1294fbd99f3">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F294F41-E2A8-4238-ADF8-3532A278FD6A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8E7618A-71E9-482D-877E-F8083117F105}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF5701D6-BC3B-45C1-94AE-8094A368E581}"/>
 </file>
</xml_diff>

<commit_message>
Changes after revisiting not executed work. Trustee portal changes properly deployed.
</commit_message>
<xml_diff>
--- a/docs/Import/FeedbackDeployment_20-09-2026.xlsx
+++ b/docs/Import/FeedbackDeployment_20-09-2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://argelisconsultancy.sharepoint.com/teams/RevitaliseRespiteHolidays/Gedeelde documenten/Optimisation Grant Application Process/Repository/Revitalise/docs/Import/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xvl/Library/CloudStorage/OneDrive-SharedLibraries-ArgelisConsultancy/Revitalise Respite Holidays - Optimisation Grant Application Process/Repository/Revitalise/docs/Import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6081984B-8EE9-7043-9DF3-2AE6DCD64D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{383A16B5-84B7-6A45-ADBA-83B7635B6303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3980" yWindow="2780" windowWidth="28040" windowHeight="17180" xr2:uid="{EDCFF76C-263F-C04F-B376-1F75C61FCC4C}"/>
+    <workbookView xWindow="1480" yWindow="780" windowWidth="33940" windowHeight="20560" xr2:uid="{EDCFF76C-263F-C04F-B376-1F75C61FCC4C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="332">
   <si>
     <t>4.1 Source 1 — Trustee Review Portal (2026-09-07)</t>
   </si>
@@ -10365,6 +10365,48 @@
   </si>
   <si>
     <t>There is a group applications table in the trustee portal. It doesn't look good. There is not enough white space bewtween the groups table and the filters under it for the individual applications. Also, it is weird to have a table, a set of filters and then another table. Create a separate screen for group applications, that is a copy of the screen for individual applications. Keeping it separate looks more clean. The group applications screen should have the screen title, the filter bar and the table with group applications. The group applications table should be removed from the application list screen so that screen only has individual applications.  When you click on an individual item of a group there is no way to navigate back to the group detail page. Make sure to correct that when building the separate group applicaitons screen. There should be an extra navigation button in the navigation bar for group applications.</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Partly done.. Income band option set not adjusted to new income band options</t>
+  </si>
+  <si>
+    <t>Not done</t>
+  </si>
+  <si>
+    <t>Done in the admin app. Not in the trustee portal yet.</t>
+  </si>
+  <si>
+    <t>Was already on the applicant table. Now also on application form but the wrong tab. Needs to be moved to general tab.</t>
+  </si>
+  <si>
+    <t>Not possible to test yet. Dependency with gravity forms export work from web builder.</t>
+  </si>
+  <si>
+    <t>not delivered</t>
+  </si>
+  <si>
+    <t>Check 25-09-2026</t>
+  </si>
+  <si>
+    <t>Partly done, see comments about the trustee role</t>
+  </si>
+  <si>
+    <t>There is a city derived column and  the wordpress to dataverse flow has new actions. Can't test it yet because of dependency web builder</t>
+  </si>
+  <si>
+    <t>Not done yet</t>
+  </si>
+  <si>
+    <t>Done last round</t>
+  </si>
+  <si>
+    <t>Not done yet.</t>
+  </si>
+  <si>
+    <t>Partly done, but not adjusted based on feedback from the 20th of September</t>
   </si>
 </sst>
 </file>
@@ -10891,1562 +10933,1674 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB4ABD2D-1E72-E244-8DDA-0B0B73A4D464}">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="65.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.83203125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="65.6640625" style="2"/>
-    <col min="3" max="3" width="27.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="29.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14" style="2" customWidth="1"/>
-    <col min="6" max="6" width="70.83203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="15.5" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="65.6640625" style="2"/>
+    <col min="1" max="1" width="25.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="65.6640625" style="2"/>
+    <col min="4" max="4" width="27.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="29.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14" style="2" customWidth="1"/>
+    <col min="7" max="7" width="70.83203125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.5" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="65.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" ht="140" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="20" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:10" ht="20" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="J2" s="12" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="76" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="171" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:10" ht="171" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="152" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:10" ht="152" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="114" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:10" ht="114" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="76" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="76" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="B8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="H8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="4" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="133" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:10" ht="133" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="38" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="I10" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="133" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:10" ht="133" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="C11" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="171" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:10" ht="171" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="G12" s="4" t="s">
+      <c r="H12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="I12" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="95" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="G13" s="4" t="s">
+      <c r="H13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="I13" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="95" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="H14" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="I14" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="40" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:10" ht="140" x14ac:dyDescent="0.2">
+      <c r="B15" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="19" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:10" ht="19" x14ac:dyDescent="0.2">
+      <c r="B16" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I16" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="76" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="4" t="s">
+      <c r="I17" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="95" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="B18" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="F18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="H18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="I18" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="38" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:10" ht="38" x14ac:dyDescent="0.2">
+      <c r="B19" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="F19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="H19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="I19" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="114" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:10" ht="114" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="G20" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="H20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="I20" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="209" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:10" ht="209" x14ac:dyDescent="0.2">
+      <c r="B21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="D21" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="F21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="H21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="I21" s="3" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="152" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:10" ht="152" x14ac:dyDescent="0.2">
+      <c r="B22" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="I22" s="3" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="76" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:10" ht="76" x14ac:dyDescent="0.2">
+      <c r="B23" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="C23" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="F23" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="H23" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="I23" s="4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="114" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
+    <row r="24" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="B24" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="C24" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="F24" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="G24" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="H24" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="I24" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="228" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:10" ht="228" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="C25" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="G25" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="H25" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="H25" s="3" t="s">
+      <c r="I25" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="95" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="C26" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="D26" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="G26" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="H26" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="3" t="s">
+      <c r="I26" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="J26" s="2" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="190" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:10" ht="190" x14ac:dyDescent="0.2">
+      <c r="B27" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="C27" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="D27" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="G27" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="H27" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H27" s="3" t="s">
+      <c r="I27" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="J27" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="57" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
+    <row r="28" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="C28" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="D28" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="G28" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="H28" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="3" t="s">
+      <c r="I28" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="114" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:10" ht="114" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="C29" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="D29" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="G29" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="H29" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="I29" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="I29" s="2" t="s">
+      <c r="J29" s="2" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="95" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+    <row r="30" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="B30" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="C30" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="D30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="E30" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E30" s="4" t="s">
+      <c r="F30" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="G30" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="H30" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H30" s="3" t="s">
+      <c r="I30" s="3" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="228" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:10" ht="228" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="C31" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="D31" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="E31" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="G31" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="G31" s="4" t="s">
+      <c r="H31" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="I31" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="95" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+    <row r="32" spans="1:10" ht="95" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="D32" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="E32" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="G32" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="G32" s="4" t="s">
+      <c r="H32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="I32" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="J32" s="2" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="114" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
+    <row r="33" spans="1:10" ht="114" x14ac:dyDescent="0.2">
+      <c r="B33" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="C33" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="D33" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="F33" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="H33" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H33" s="3" t="s">
+      <c r="I33" s="3" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="190" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+    <row r="34" spans="1:10" ht="190" x14ac:dyDescent="0.2">
+      <c r="A34" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B34" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="F34" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="G34" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="H34" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H34" s="3" t="s">
+      <c r="I34" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="J34" s="2" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="57" x14ac:dyDescent="0.2">
-      <c r="A35" s="3" t="s">
+    <row r="35" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="B35" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="C35" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="D35" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E35" s="4" t="s">
+      <c r="F35" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="G35" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="H35" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="I35" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
+    <row r="36" spans="1:10" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A36" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B36" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="C36" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="H36" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="I36" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="J36" s="2" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="209" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
+    <row r="37" spans="1:10" ht="209" x14ac:dyDescent="0.2">
+      <c r="B37" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="C37" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="F37" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="G37" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="H37" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H37" s="10" t="s">
+      <c r="I37" s="10" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="209" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
+    <row r="38" spans="1:10" ht="209" x14ac:dyDescent="0.2">
+      <c r="A38" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="C38" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="D38" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="F38" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="G38" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="H38" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="I38" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="152" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
+    <row r="39" spans="1:10" ht="152" x14ac:dyDescent="0.2">
+      <c r="A39" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="C39" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="D39" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="E39" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="F39" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="G39" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="H39" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="H39" s="3" t="s">
+      <c r="I39" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="J39" s="2" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="228" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
+    <row r="40" spans="1:10" ht="228" x14ac:dyDescent="0.2">
+      <c r="A40" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B40" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B40" s="4" t="s">
+      <c r="C40" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="D40" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="E40" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="F40" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="I40" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="J40" s="2" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="247" x14ac:dyDescent="0.2">
-      <c r="A41" s="3" t="s">
+    <row r="41" spans="1:10" ht="247" x14ac:dyDescent="0.2">
+      <c r="A41" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B41" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="C41" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="D41" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="F41" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="G41" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="H41" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="I41" s="3" t="s">
         <v>237</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="266" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
+    <row r="42" spans="1:10" ht="266" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B42" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="C42" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="D42" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="F42" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="G42" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="H42" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="I42" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="57" x14ac:dyDescent="0.2">
-      <c r="A43" s="3" t="s">
+    <row r="43" spans="1:10" ht="187" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="B43" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="C43" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="D43" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="F43" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="G43" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="H43" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H43" s="4" t="s">
+      <c r="I43" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="57" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
+    <row r="44" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="C44" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="D44" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="E44" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E44" s="3" t="s">
+      <c r="F44" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="G44" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="G44" s="4" t="s">
+      <c r="H44" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H44" s="3" t="s">
+      <c r="I44" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="J44" s="2" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="40" x14ac:dyDescent="0.2">
-      <c r="A45" s="1" t="s">
+    <row r="45" spans="1:10" ht="140" x14ac:dyDescent="0.2">
+      <c r="B45" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="19" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
+    <row r="46" spans="1:10" ht="19" x14ac:dyDescent="0.2">
+      <c r="B46" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="C46" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C46" s="3" t="s">
+      <c r="D46" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="E46" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E46" s="3" t="s">
+      <c r="F46" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="G46" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G46" s="3" t="s">
+      <c r="H46" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H46" s="3" t="s">
+      <c r="I46" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="323" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
+    <row r="47" spans="1:10" ht="323" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="C47" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="C47" s="4" t="s">
+      <c r="D47" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D47" s="11" t="s">
+      <c r="E47" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="E47" s="3" t="s">
+      <c r="F47" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F47" s="3" t="s">
+      <c r="G47" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="G47" s="3" t="s">
+      <c r="H47" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="H47" s="3" t="s">
+      <c r="I47" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="I47" s="2" t="s">
+      <c r="J47" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
+    <row r="48" spans="1:10" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A48" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="C48" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="D48" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="E48" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E48" s="4" t="s">
+      <c r="F48" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="G48" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="G48" s="3" t="s">
+      <c r="H48" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H48" s="3" t="s">
+      <c r="I48" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="J48" s="2" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="266" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
+    <row r="49" spans="1:10" ht="266" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B49" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="C49" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="D49" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D49" s="5" t="s">
+      <c r="E49" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E49" s="3" t="s">
+      <c r="F49" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="G49" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="G49" s="4" t="s">
+      <c r="H49" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H49" s="3" t="s">
+      <c r="I49" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="J49" s="2" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="342" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
+    <row r="50" spans="1:10" ht="342" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B50" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="C50" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="D50" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="E50" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E50" s="4" t="s">
+      <c r="F50" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="G50" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="G50" s="3" t="s">
+      <c r="H50" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="H50" s="3" t="s">
+      <c r="I50" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="I50" s="2" t="s">
+      <c r="J50" s="2" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="133" x14ac:dyDescent="0.2">
-      <c r="A51" s="3" t="s">
+    <row r="51" spans="1:10" ht="133" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="C51" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="C51" s="4" t="s">
+      <c r="D51" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="E51" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E51" s="3" t="s">
+      <c r="F51" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="G51" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G51" s="3" t="s">
+      <c r="H51" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H51" s="3" t="s">
+      <c r="I51" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="I51" s="2" t="s">
+      <c r="J51" s="2" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="247" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
+    <row r="52" spans="1:10" ht="247" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="C52" s="4" t="s">
         <v>261</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="D52" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="E52" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E52" s="3" t="s">
+      <c r="F52" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F52" s="3" t="s">
+      <c r="G52" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="G52" s="4" t="s">
+      <c r="H52" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H52" s="3" t="s">
+      <c r="I52" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="I52" s="2" t="s">
+      <c r="J52" s="2" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="247" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
+    <row r="53" spans="1:10" ht="247" x14ac:dyDescent="0.2">
+      <c r="B53" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="C53" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="D53" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="E53" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="E53" s="3" t="s">
+      <c r="F53" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="F53" s="3" t="s">
+      <c r="G53" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="G53" s="4" t="s">
+      <c r="H53" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H53" s="3" t="s">
+      <c r="I53" s="3" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="20" x14ac:dyDescent="0.2">
-      <c r="A54" s="1" t="s">
+    <row r="54" spans="1:10" ht="40" x14ac:dyDescent="0.2">
+      <c r="B54" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="169" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
+    <row r="55" spans="1:10" ht="169" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="3" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="19" x14ac:dyDescent="0.2">
-      <c r="A56" s="3" t="s">
+    <row r="56" spans="1:10" ht="19" x14ac:dyDescent="0.2">
+      <c r="B56" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="C56" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="D56" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D56" s="3" t="s">
+      <c r="E56" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="F56" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F56" s="3" t="s">
+      <c r="G56" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G56" s="3" t="s">
+      <c r="H56" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H56" s="3" t="s">
+      <c r="I56" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="57" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
+    <row r="57" spans="1:10" ht="57" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="C57" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="C57" s="4" t="s">
+      <c r="D57" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D57" s="5" t="s">
+      <c r="E57" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E57" s="3" t="s">
+      <c r="F57" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F57" s="3" t="s">
+      <c r="G57" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="G57" s="3" t="s">
+      <c r="H57" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="H57" s="3" t="s">
+      <c r="I57" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="I57" s="2" t="s">
+      <c r="J57" s="2" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="342" x14ac:dyDescent="0.2">
-      <c r="A58" s="3" t="s">
+    <row r="58" spans="1:10" ht="342" x14ac:dyDescent="0.2">
+      <c r="B58" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="C58" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="C58" s="4" t="s">
+      <c r="D58" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="D58" s="3" t="s">
+      <c r="E58" s="3" t="s">
         <v>273</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="F58" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="F58" s="3" t="s">
+      <c r="G58" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="G58" s="4" t="s">
+      <c r="H58" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H58" s="3" t="s">
+      <c r="I58" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="I58" s="2" t="s">
+      <c r="J58" s="2" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="114" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
+    <row r="59" spans="1:10" ht="114" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="C59" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="D59" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D59" s="5" t="s">
+      <c r="E59" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="F59" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="G59" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="G59" s="4" t="s">
+      <c r="H59" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H59" s="3" t="s">
+      <c r="I59" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="I59" s="2" t="s">
+      <c r="J59" s="2" t="s">
         <v>307</v>
       </c>
     </row>
@@ -12456,6 +12610,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae75f7d6110eb3c01e30b5864ecce8d9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" xmlns:ns3="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f758225586994ab2ed7147b7dc97d7e" ns2:_="" ns3:_="">
     <xsd:import namespace="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
@@ -12636,34 +12810,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F294F41-E2A8-4238-ADF8-3532A278FD6A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF5701D6-BC3B-45C1-94AE-8094A368E581}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
+    <ds:schemaRef ds:uri="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8E7618A-71E9-482D-877E-F8083117F105}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C8E7618A-71E9-482D-877E-F8083117F105}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF5701D6-BC3B-45C1-94AE-8094A368E581}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F294F41-E2A8-4238-ADF8-3532A278FD6A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
+    <ds:schemaRef ds:uri="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>